<commit_message>
MAJ tarif via Power Automate
</commit_message>
<xml_diff>
--- a/data/TarifVinom_Master.xlsx
+++ b/data/TarifVinom_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sfrbt1009862.sharepoint.com/vinom/Shared Documents/TARIF VINOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{641ED796-E10E-4877-96BF-4A71D8601ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C74DB958-37A5-C44A-864A-CA43B4AA3EAA}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{641ED796-E10E-4877-96BF-4A71D8601ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F57E1C8-5856-084C-9E76-56E3D282B874}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="23260" windowHeight="12460" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10712" uniqueCount="2245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10710" uniqueCount="2245">
   <si>
     <t>TARIF VINOM MASTER — Document de pilotage du catalogue automatisé</t>
   </si>
@@ -18482,8 +18482,8 @@
       </c>
     </row>
     <row r="275" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A275" t="s">
-        <v>806</v>
+      <c r="A275">
+        <v>43800825</v>
       </c>
       <c r="B275" t="s">
         <v>56</v>
@@ -18509,8 +18509,8 @@
       <c r="I275" t="s">
         <v>62</v>
       </c>
-      <c r="J275" t="s">
-        <v>94</v>
+      <c r="J275">
+        <v>2025</v>
       </c>
       <c r="K275">
         <v>75</v>
@@ -49315,6 +49315,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="8b06e530-ed80-4ff0-be41-2806c2470479" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ee8e01a-5661-48eb-b75f-361470a34d5b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010002F00E183A222D47876A51DABA610BDE" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="860f336250d6f7d113c3b43983ff209d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ee8e01a-5661-48eb-b75f-361470a34d5b" xmlns:ns3="a1e62e11-0de7-4d84-85a0-444df097221b" xmlns:ns4="8b06e530-ed80-4ff0-be41-2806c2470479" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f4eda2c29f4341f43b2cc38e2775c30" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="3ee8e01a-5661-48eb-b75f-361470a34d5b"/>
@@ -49574,17 +49585,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="8b06e530-ed80-4ff0-be41-2806c2470479" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ee8e01a-5661-48eb-b75f-361470a34d5b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -49595,6 +49595,24 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DE35E19-146F-4A5C-934B-8F843242C74E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="3ee8e01a-5661-48eb-b75f-361470a34d5b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="a1e62e11-0de7-4d84-85a0-444df097221b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8b06e530-ed80-4ff0-be41-2806c2470479"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A2293BB-1BB0-48A0-A955-B37D029329BC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -49614,24 +49632,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DE35E19-146F-4A5C-934B-8F843242C74E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="8b06e530-ed80-4ff0-be41-2806c2470479"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3ee8e01a-5661-48eb-b75f-361470a34d5b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a1e62e11-0de7-4d84-85a0-444df097221b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0FE2C01-6340-45D6-8526-0AB30AB8259E}">
   <ds:schemaRefs>

</xml_diff>